<commit_message>
Added SimpleQuantity, Range, Ratio, ServiceRequest
</commit_message>
<xml_diff>
--- a/314e-ig/output/CodeSystem-attachment-tag.xlsx
+++ b/314e-ig/output/CodeSystem-attachment-tag.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-05-15T09:21:03+05:30</t>
+    <t>2026-05-16T07:30:07+05:30</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -141,7 +141,7 @@
     <t>inline-data-externalized-to-file</t>
   </si>
   <si>
-    <t>Inline data externalized to and saved as file</t>
+    <t>Inline data externalized and saved as file</t>
   </si>
   <si>
     <t>Indicates that the Attachment content was originally available

</xml_diff>